<commit_message>
feat: Offline Data Lake mimarisi, merkezi komisyon (fees) sistemi ve yeni stratejiler (90+) eklendi
</commit_message>
<xml_diff>
--- a/vbt_bist/output/AEFES/AEFES_Karsilastirma.xlsx
+++ b/vbt_bist/output/AEFES/AEFES_Karsilastirma.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,11 +441,11 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>hist_vol</t>
+          <t>rsi_divergence</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>34.25</v>
+        <v>60.72</v>
       </c>
     </row>
     <row r="3">
@@ -456,11 +456,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>three_ma</t>
+          <t>ultimate_osc</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>21.63</v>
+        <v>53.12</v>
       </c>
     </row>
     <row r="4">
@@ -471,11 +471,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>supertrend</t>
+          <t>hist_vol</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>18.59</v>
+        <v>34.25</v>
       </c>
     </row>
     <row r="5">
@@ -486,11 +486,11 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>cmo</t>
+          <t>historical_vol_rank</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>15.08</v>
+        <v>34.23</v>
       </c>
     </row>
     <row r="6">
@@ -501,11 +501,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>rsi</t>
+          <t>golden_cross</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>13.68</v>
+        <v>33.55</v>
       </c>
     </row>
     <row r="7">
@@ -516,11 +516,11 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>donchian</t>
+          <t>three_ma</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>9.970000000000001</v>
+        <v>21.63</v>
       </c>
     </row>
     <row r="8">
@@ -531,11 +531,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>single_ma</t>
+          <t>schaff_trend</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>9.029999999999999</v>
+        <v>20.81</v>
       </c>
     </row>
     <row r="9">
@@ -546,11 +546,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>cmf</t>
+          <t>obv_ma</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>7.02</v>
+        <v>18.79</v>
       </c>
     </row>
     <row r="10">
@@ -561,11 +561,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>macd</t>
+          <t>supertrend</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>6.86</v>
+        <v>18.59</v>
       </c>
     </row>
     <row r="11">
@@ -576,11 +576,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>inside_bar</t>
+          <t>pin_bar</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>6.63</v>
+        <v>18.15</v>
       </c>
     </row>
     <row r="12">
@@ -591,11 +591,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>fractal_breakout</t>
+          <t>dpo</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>4.96</v>
+        <v>16.74</v>
       </c>
     </row>
     <row r="13">
@@ -606,11 +606,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>doji_reversal</t>
+          <t>vwap</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>4.04</v>
+        <v>16.52</v>
       </c>
     </row>
     <row r="14">
@@ -621,11 +621,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>coppock</t>
+          <t>cmo</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>15.08</v>
       </c>
     </row>
     <row r="15">
@@ -636,11 +636,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>engulfing</t>
+          <t>rsi</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>13.68</v>
       </c>
     </row>
     <row r="16">
@@ -651,11 +651,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>vpt</t>
+          <t>donchian</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>-0.18</v>
+        <v>9.970000000000001</v>
       </c>
     </row>
     <row r="17">
@@ -666,11 +666,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>cci</t>
+          <t>single_ma</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>-0.79</v>
+        <v>9.029999999999999</v>
       </c>
     </row>
     <row r="18">
@@ -681,11 +681,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>williams_r</t>
+          <t>cmf</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>-1.14</v>
+        <v>7.02</v>
       </c>
     </row>
     <row r="19">
@@ -696,11 +696,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>kst</t>
+          <t>macd</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>-3.13</v>
+        <v>6.86</v>
       </c>
     </row>
     <row r="20">
@@ -711,11 +711,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>two_ma</t>
+          <t>inside_bar</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>-3.81</v>
+        <v>6.63</v>
       </c>
     </row>
     <row r="21">
@@ -726,11 +726,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>mfi</t>
+          <t>atr_channel</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>-4.53</v>
+        <v>6.34</v>
       </c>
     </row>
     <row r="22">
@@ -741,11 +741,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>hma</t>
+          <t>fractal_breakout</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>-5.13</v>
+        <v>4.96</v>
       </c>
     </row>
     <row r="23">
@@ -756,11 +756,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>stochastic</t>
+          <t>doji_reversal</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>-7.12</v>
+        <v>4.04</v>
       </c>
     </row>
     <row r="24">
@@ -771,11 +771,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ichimoku</t>
+          <t>connors_rsi</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>-9.130000000000001</v>
+        <v>3.54</v>
       </c>
     </row>
     <row r="25">
@@ -786,11 +786,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>adx</t>
+          <t>chandelier</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>-9.369999999999999</v>
+        <v>0.37</v>
       </c>
     </row>
     <row r="26">
@@ -801,11 +801,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>awesome_oscillator</t>
+          <t>pvi</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>-9.619999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -816,11 +816,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>tsi</t>
+          <t>vpt</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>-11.12</v>
+        <v>-0.18</v>
       </c>
     </row>
     <row r="28">
@@ -831,11 +831,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>zscore</t>
+          <t>cci</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>-12.57</v>
+        <v>-0.79</v>
       </c>
     </row>
     <row r="29">
@@ -846,11 +846,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>tema</t>
+          <t>williams_r</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>-13.57</v>
+        <v>-1.14</v>
       </c>
     </row>
     <row r="30">
@@ -861,11 +861,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>bollinger</t>
+          <t>natr</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>-14.25</v>
+        <v>-2.01</v>
       </c>
     </row>
     <row r="31">
@@ -876,11 +876,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>alma</t>
+          <t>coppock</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>-15.54</v>
+        <v>-2.3</v>
       </c>
     </row>
     <row r="32">
@@ -891,11 +891,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>keltner</t>
+          <t>nvi</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>-20.06</v>
+        <v>-2.57</v>
       </c>
     </row>
     <row r="33">
@@ -906,11 +906,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>mean_reversion</t>
+          <t>kst</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>-20.51</v>
+        <v>-3.13</v>
       </c>
     </row>
     <row r="34">
@@ -921,11 +921,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>std_channel</t>
+          <t>two_ma</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>-21.62</v>
+        <v>-3.81</v>
       </c>
     </row>
     <row r="35">
@@ -936,11 +936,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>wma</t>
+          <t>mfi</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>-22.38</v>
+        <v>-4.53</v>
       </c>
     </row>
     <row r="36">
@@ -951,11 +951,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>psar</t>
+          <t>hma</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>-22.44</v>
+        <v>-5.13</v>
       </c>
     </row>
     <row r="37">
@@ -966,11 +966,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>obv</t>
+          <t>marubozu</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>-26.68</v>
+        <v>-5.33</v>
       </c>
     </row>
     <row r="38">
@@ -981,11 +981,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>linreg</t>
+          <t>awesome_oscillator</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>-27.16</v>
+        <v>-5.51</v>
       </c>
     </row>
     <row r="39">
@@ -996,11 +996,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>aroon</t>
+          <t>trix</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>-28</v>
+        <v>-6.38</v>
       </c>
     </row>
     <row r="40">
@@ -1011,11 +1011,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>roc</t>
+          <t>stochastic</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>-31.7</v>
+        <v>-7.12</v>
       </c>
     </row>
     <row r="41">
@@ -1026,10 +1026,535 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
+          <t>klinger</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>-7.65</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>momentum</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>-8.69</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>bb_width</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>-8.779999999999999</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>ichimoku</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>-9.130000000000001</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>adx</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>-9.369999999999999</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>stoch_rsi</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>-10.57</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>tsi</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>-11.12</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>ema_cross</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>-11.13</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>heikin_ashi</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>-11.65</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>zscore</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>-12.57</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>hammer</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>-12.74</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>tema</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>-13.57</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>supertrend_rsi</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>-14.1</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>bollinger</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>-14.25</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>alma</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>-15.54</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>ad_line</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>-16.12</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>squeeze</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>-17.01</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>rainbow_ma</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>-18.45</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>keltner</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>-20.06</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>engulfing</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>-20.34</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>mean_reversion</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>-20.51</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>std_channel</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>-21.62</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>wma</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>-22.38</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>psar</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>-22.44</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>dema</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>-22.68</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>true_range_ema</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>-26.37</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>obv</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>-26.68</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>linreg</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>-27.16</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>aroon</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>-28</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>zlema</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>-30</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>trend_intensity</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>-30.14</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>three_soldiers</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>-31.07</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>ichimoku_rsi</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>-31.39</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>roc</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>-31.7</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>rsi_macd</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>-31.93</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>AEFES</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
           <t>vix_fix</t>
         </is>
       </c>
-      <c r="C41" t="n">
+      <c r="C76" t="n">
         <v>-33.66</v>
       </c>
     </row>

</xml_diff>